<commit_message>
fix(opkom): fix branch code mapping across all branches so service values like Sorong Rupa-Rupa match input data
</commit_message>
<xml_diff>
--- a/data/input_data.xlsx
+++ b/data/input_data.xlsx
@@ -10501,7 +10501,7 @@
         <v>9</v>
       </c>
       <c r="C6" t="str">
-        <v>R02</v>
+        <v>R01</v>
       </c>
       <c r="D6" t="str">
         <v>Makassar</v>
@@ -10637,7 +10637,7 @@
         <v>9</v>
       </c>
       <c r="C11" t="str">
-        <v>R03</v>
+        <v>R02</v>
       </c>
       <c r="D11" t="str">
         <v>TPK Makassar</v>
@@ -10779,7 +10779,7 @@
         <v>9</v>
       </c>
       <c r="C16" t="str">
-        <v>R04</v>
+        <v>R03</v>
       </c>
       <c r="D16" t="str">
         <v>Samarinda</v>
@@ -11069,7 +11069,7 @@
         <v>9</v>
       </c>
       <c r="C26" t="str">
-        <v>R06</v>
+        <v>R05</v>
       </c>
       <c r="D26" t="str">
         <v>Bitung</v>
@@ -11205,7 +11205,7 @@
         <v>9</v>
       </c>
       <c r="C31" t="str">
-        <v>R07</v>
+        <v>R06</v>
       </c>
       <c r="D31" t="str">
         <v>TPK Bitung</v>
@@ -11347,7 +11347,7 @@
         <v>9</v>
       </c>
       <c r="C36" t="str">
-        <v>R08</v>
+        <v>R07</v>
       </c>
       <c r="D36" t="str">
         <v>Ambon</v>
@@ -11492,7 +11492,7 @@
         <v>9</v>
       </c>
       <c r="C41" t="str">
-        <v>R09</v>
+        <v>R08</v>
       </c>
       <c r="D41" t="str">
         <v>Sorong</v>
@@ -11637,7 +11637,7 @@
         <v>9</v>
       </c>
       <c r="C46" t="str">
-        <v>R10</v>
+        <v>R09</v>
       </c>
       <c r="D46" t="str">
         <v>Jayapura</v>
@@ -11782,7 +11782,7 @@
         <v>9</v>
       </c>
       <c r="C51" t="str">
-        <v>R11</v>
+        <v>R10</v>
       </c>
       <c r="D51" t="str">
         <v>Tarakan</v>
@@ -11927,7 +11927,7 @@
         <v>9</v>
       </c>
       <c r="C56" t="str">
-        <v>R12</v>
+        <v>R11</v>
       </c>
       <c r="D56" t="str">
         <v>Pantoloan</v>
@@ -12072,7 +12072,7 @@
         <v>9</v>
       </c>
       <c r="C61" t="str">
-        <v>R13</v>
+        <v>R12</v>
       </c>
       <c r="D61" t="str">
         <v>Ternate</v>
@@ -12217,7 +12217,7 @@
         <v>9</v>
       </c>
       <c r="C66" t="str">
-        <v>R14</v>
+        <v>R13</v>
       </c>
       <c r="D66" t="str">
         <v>Kendari</v>
@@ -12362,7 +12362,7 @@
         <v>9</v>
       </c>
       <c r="C71" t="str">
-        <v>R15</v>
+        <v>R14</v>
       </c>
       <c r="D71" t="str">
         <v>Parepare</v>
@@ -12507,7 +12507,7 @@
         <v>9</v>
       </c>
       <c r="C76" t="str">
-        <v>R16</v>
+        <v>R15</v>
       </c>
       <c r="D76" t="str">
         <v>Biak</v>
@@ -12652,7 +12652,7 @@
         <v>9</v>
       </c>
       <c r="C81" t="str">
-        <v>R17</v>
+        <v>R16</v>
       </c>
       <c r="D81" t="str">
         <v>Merauke</v>
@@ -12797,7 +12797,7 @@
         <v>9</v>
       </c>
       <c r="C86" t="str">
-        <v>R18</v>
+        <v>R17</v>
       </c>
       <c r="D86" t="str">
         <v>Manokwari</v>
@@ -12942,7 +12942,7 @@
         <v>9</v>
       </c>
       <c r="C91" t="str">
-        <v>R19</v>
+        <v>R18</v>
       </c>
       <c r="D91" t="str">
         <v>Nunukan</v>
@@ -13087,7 +13087,7 @@
         <v>9</v>
       </c>
       <c r="C96" t="str">
-        <v>R20</v>
+        <v>R19</v>
       </c>
       <c r="D96" t="str">
         <v>Tg Redeb</v>
@@ -13232,7 +13232,7 @@
         <v>9</v>
       </c>
       <c r="C101" t="str">
-        <v>R21</v>
+        <v>R20</v>
       </c>
       <c r="D101" t="str">
         <v>Gorontalo</v>
@@ -13377,7 +13377,7 @@
         <v>9</v>
       </c>
       <c r="C106" t="str">
-        <v>R22</v>
+        <v>R21</v>
       </c>
       <c r="D106" t="str">
         <v>Fakfak</v>
@@ -13522,7 +13522,7 @@
         <v>9</v>
       </c>
       <c r="C111" t="str">
-        <v>R23</v>
+        <v>R22</v>
       </c>
       <c r="D111" t="str">
         <v>Tolitoli</v>
@@ -13667,7 +13667,7 @@
         <v>9</v>
       </c>
       <c r="C116" t="str">
-        <v>R24</v>
+        <v>R23</v>
       </c>
       <c r="D116" t="str">
         <v>Manado</v>
@@ -13803,7 +13803,7 @@
         <v>9</v>
       </c>
       <c r="C121" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D121" t="str">
         <v>Makassar New Port</v>
@@ -13945,7 +13945,7 @@
         <v>9</v>
       </c>
       <c r="C126" t="str">
-        <v>R26</v>
+        <v>R25</v>
       </c>
       <c r="D126" t="str">
         <v xml:space="preserve">Bontang  </v>
@@ -14078,7 +14078,7 @@
         <v>9</v>
       </c>
       <c r="C131" t="str">
-        <v>R27</v>
+        <v>R26</v>
       </c>
       <c r="D131" t="str">
         <v>KKT</v>
@@ -38789,7 +38789,7 @@
         <v>9</v>
       </c>
       <c r="C463" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D463" t="str">
         <v>Makassar New Port</v>
@@ -38821,7 +38821,7 @@
         <v>9</v>
       </c>
       <c r="C464" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D464" t="str">
         <v>Makassar New Port</v>
@@ -38847,7 +38847,7 @@
         <v>9</v>
       </c>
       <c r="C465" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D465" t="str">
         <v>Makassar New Port</v>
@@ -38873,7 +38873,7 @@
         <v>9</v>
       </c>
       <c r="C466" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D466" t="str">
         <v>Makassar New Port</v>
@@ -38905,7 +38905,7 @@
         <v>9</v>
       </c>
       <c r="C467" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D467" t="str">
         <v>Makassar New Port</v>
@@ -38937,7 +38937,7 @@
         <v>9</v>
       </c>
       <c r="C468" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D468" t="str">
         <v>Makassar New Port</v>
@@ -38969,7 +38969,7 @@
         <v>9</v>
       </c>
       <c r="C469" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D469" t="str">
         <v>Makassar New Port</v>
@@ -38995,7 +38995,7 @@
         <v>9</v>
       </c>
       <c r="C470" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D470" t="str">
         <v>Makassar New Port</v>
@@ -39021,7 +39021,7 @@
         <v>9</v>
       </c>
       <c r="C471" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D471" t="str">
         <v>Makassar New Port</v>
@@ -39050,7 +39050,7 @@
         <v>9</v>
       </c>
       <c r="C472" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D472" t="str">
         <v>Makassar New Port</v>
@@ -39079,7 +39079,7 @@
         <v>9</v>
       </c>
       <c r="C473" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D473" t="str">
         <v>Makassar New Port</v>
@@ -39105,7 +39105,7 @@
         <v>9</v>
       </c>
       <c r="C474" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D474" t="str">
         <v>Makassar New Port</v>
@@ -39131,7 +39131,7 @@
         <v>9</v>
       </c>
       <c r="C475" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D475" t="str">
         <v>Makassar New Port</v>
@@ -39157,7 +39157,7 @@
         <v>9</v>
       </c>
       <c r="C476" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D476" t="str">
         <v>Makassar New Port</v>
@@ -39183,7 +39183,7 @@
         <v>9</v>
       </c>
       <c r="C477" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D477" t="str">
         <v>Makassar New Port</v>
@@ -39209,7 +39209,7 @@
         <v>9</v>
       </c>
       <c r="C478" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D478" t="str">
         <v>Makassar New Port</v>
@@ -39238,7 +39238,7 @@
         <v>9</v>
       </c>
       <c r="C479" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D479" t="str">
         <v>Makassar New Port</v>
@@ -39264,7 +39264,7 @@
         <v>9</v>
       </c>
       <c r="C480" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D480" t="str">
         <v>Makassar New Port</v>
@@ -39290,7 +39290,7 @@
         <v>9</v>
       </c>
       <c r="C481" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D481" t="str">
         <v>Makassar New Port</v>
@@ -39316,7 +39316,7 @@
         <v>9</v>
       </c>
       <c r="C482" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D482" t="str">
         <v>Makassar New Port</v>
@@ -39342,7 +39342,7 @@
         <v>9</v>
       </c>
       <c r="C483" t="str">
-        <v>R25</v>
+        <v>R24</v>
       </c>
       <c r="D483" t="str">
         <v>Makassar New Port</v>

</xml_diff>